<commit_message>
feat: afegir recompte registrades/esperades al resum de correccions
- modules/correccio.py: emmagatzema `counts` (n01–n06, ref_compres, ref_vendes) per alumne a resultats.json
- views/professor/correccio.py: taula resum renderitzada com a HTML pur (_taula_resum_html) amb columnes Comandes/Recepcions/Factures centrades i color taronja quan registrades ≠ esperades; Penalització a 2 decimals
- CLAUDE.md: documentada la decisió de disseny (st.dataframe no suporta text-align)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/tasques/02.20/ADG32/entregues/6478/02.20-6478-03_FACTURES_COMPRA.xlsx
+++ b/data/tasques/02.20/ADG32/entregues/6478/02.20-6478-03_FACTURES_COMPRA.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="295">
   <si>
     <t>Número</t>
   </si>
@@ -653,6 +653,252 @@
   </si>
   <si>
     <t>26588596</t>
+  </si>
+  <si>
+    <t>FC/2025/0037</t>
+  </si>
+  <si>
+    <t>26588615</t>
+  </si>
+  <si>
+    <t>FC/2025/0036</t>
+  </si>
+  <si>
+    <t>26588633</t>
+  </si>
+  <si>
+    <t>FC/2025/0033</t>
+  </si>
+  <si>
+    <t>2025/00023</t>
+  </si>
+  <si>
+    <t>C-C/00014</t>
+  </si>
+  <si>
+    <t>FC/2025/0032</t>
+  </si>
+  <si>
+    <t>2025/00021</t>
+  </si>
+  <si>
+    <t>C-C/00013</t>
+  </si>
+  <si>
+    <t>FC/2025/0020</t>
+  </si>
+  <si>
+    <t>2025/00017</t>
+  </si>
+  <si>
+    <t>C-C/00012</t>
+  </si>
+  <si>
+    <t>FC/2025/0019</t>
+  </si>
+  <si>
+    <t>2025/00019</t>
+  </si>
+  <si>
+    <t>C-C/00011</t>
+  </si>
+  <si>
+    <t>FC/2025/0031</t>
+  </si>
+  <si>
+    <t>0026469156</t>
+  </si>
+  <si>
+    <t>FC/2025/0030</t>
+  </si>
+  <si>
+    <t>0026469138</t>
+  </si>
+  <si>
+    <t>FC/2025/0029</t>
+  </si>
+  <si>
+    <t>026469119</t>
+  </si>
+  <si>
+    <t>FC/2025/0028</t>
+  </si>
+  <si>
+    <t>0026387171</t>
+  </si>
+  <si>
+    <t>FC/2025/0027</t>
+  </si>
+  <si>
+    <t>0026387132</t>
+  </si>
+  <si>
+    <t>FC/2025/0026</t>
+  </si>
+  <si>
+    <t>0026387152</t>
+  </si>
+  <si>
+    <t>FC/2025/0010</t>
+  </si>
+  <si>
+    <t>2025/00014</t>
+  </si>
+  <si>
+    <t>C-C/00010</t>
+  </si>
+  <si>
+    <t>FC/2025/0009</t>
+  </si>
+  <si>
+    <t>C-C/00009</t>
+  </si>
+  <si>
+    <t>FC/2025/0008</t>
+  </si>
+  <si>
+    <t>2025/00009</t>
+  </si>
+  <si>
+    <t>C-C/00007</t>
+  </si>
+  <si>
+    <t>FC/2025/0007</t>
+  </si>
+  <si>
+    <t>2025/00010</t>
+  </si>
+  <si>
+    <t>C-C/00008</t>
+  </si>
+  <si>
+    <t>FC/2025/0025</t>
+  </si>
+  <si>
+    <t>0026311626</t>
+  </si>
+  <si>
+    <t>FC/2025/0024</t>
+  </si>
+  <si>
+    <t>0026311607</t>
+  </si>
+  <si>
+    <t>FC/2025/0023</t>
+  </si>
+  <si>
+    <t>0026311586</t>
+  </si>
+  <si>
+    <t>FC/2025/0022</t>
+  </si>
+  <si>
+    <t>1038746</t>
+  </si>
+  <si>
+    <t>FC/2025/0021</t>
+  </si>
+  <si>
+    <t>1037825</t>
+  </si>
+  <si>
+    <t>FC/2025/0018</t>
+  </si>
+  <si>
+    <t>0026258069</t>
+  </si>
+  <si>
+    <t>FC/2025/0017</t>
+  </si>
+  <si>
+    <t>0026258049</t>
+  </si>
+  <si>
+    <t>FC/2025/0014</t>
+  </si>
+  <si>
+    <t>1035426</t>
+  </si>
+  <si>
+    <t>FC/2025/0016</t>
+  </si>
+  <si>
+    <t>0026247317</t>
+  </si>
+  <si>
+    <t>FC/2025/0006</t>
+  </si>
+  <si>
+    <t>2025/00008</t>
+  </si>
+  <si>
+    <t>C-C/00006</t>
+  </si>
+  <si>
+    <t>FC/2025/0005</t>
+  </si>
+  <si>
+    <t>C-C/00005</t>
+  </si>
+  <si>
+    <t>FC/2025/0015</t>
+  </si>
+  <si>
+    <t>0026189546</t>
+  </si>
+  <si>
+    <t>FC/2025/0004</t>
+  </si>
+  <si>
+    <t>2025/00006</t>
+  </si>
+  <si>
+    <t>C-C/00004</t>
+  </si>
+  <si>
+    <t>FC/2025/0003</t>
+  </si>
+  <si>
+    <t>2025/00004</t>
+  </si>
+  <si>
+    <t>C-C/00003</t>
+  </si>
+  <si>
+    <t>FC/2025/0002</t>
+  </si>
+  <si>
+    <t>2025/00001</t>
+  </si>
+  <si>
+    <t>C-C/00001</t>
+  </si>
+  <si>
+    <t>FC/2025/0001</t>
+  </si>
+  <si>
+    <t>2025/00005</t>
+  </si>
+  <si>
+    <t>C-C/00002</t>
+  </si>
+  <si>
+    <t>FC/2025/0013</t>
+  </si>
+  <si>
+    <t>1026885</t>
+  </si>
+  <si>
+    <t>FC/2025/0012</t>
+  </si>
+  <si>
+    <t>1026251</t>
+  </si>
+  <si>
+    <t>FC/2025/0011</t>
+  </si>
+  <si>
+    <t>1024608</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1252,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="30.7109375" customWidth="1"/>
@@ -3490,6 +3736,1084 @@
         <v>13</v>
       </c>
     </row>
+    <row r="82" spans="1:10">
+      <c r="A82" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D82" s="3">
+        <v>45989</v>
+      </c>
+      <c r="E82" s="3">
+        <v>45989</v>
+      </c>
+      <c r="F82" s="2"/>
+      <c r="G82" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H82" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I82" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J82" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10">
+      <c r="A83" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D83" s="3">
+        <v>45989</v>
+      </c>
+      <c r="E83" s="3">
+        <v>45989</v>
+      </c>
+      <c r="F83" s="2"/>
+      <c r="G83" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H83" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I83" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10">
+      <c r="A84" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D84" s="3">
+        <v>45987</v>
+      </c>
+      <c r="E84" s="3">
+        <v>45994</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="G84" s="4">
+        <v>-3126</v>
+      </c>
+      <c r="H84" s="4">
+        <v>-656.46</v>
+      </c>
+      <c r="I84" s="4">
+        <v>-3782.46</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10">
+      <c r="A85" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D85" s="3">
+        <v>45987</v>
+      </c>
+      <c r="E85" s="3">
+        <v>45994</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G85" s="4">
+        <v>-3704</v>
+      </c>
+      <c r="H85" s="4">
+        <v>-777.84</v>
+      </c>
+      <c r="I85" s="4">
+        <v>-4481.84</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10">
+      <c r="A86" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D86" s="3">
+        <v>45981</v>
+      </c>
+      <c r="E86" s="3">
+        <v>45988</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G86" s="4">
+        <v>-3107</v>
+      </c>
+      <c r="H86" s="4">
+        <v>-652.47</v>
+      </c>
+      <c r="I86" s="4">
+        <v>-3759.47</v>
+      </c>
+      <c r="J86" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10">
+      <c r="A87" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D87" s="3">
+        <v>45981</v>
+      </c>
+      <c r="E87" s="3">
+        <v>45988</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G87" s="4">
+        <v>-2712</v>
+      </c>
+      <c r="H87" s="4">
+        <v>-569.52</v>
+      </c>
+      <c r="I87" s="4">
+        <v>-3281.52</v>
+      </c>
+      <c r="J87" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10">
+      <c r="A88" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D88" s="3">
+        <v>45980</v>
+      </c>
+      <c r="E88" s="3">
+        <v>45980</v>
+      </c>
+      <c r="F88" s="2"/>
+      <c r="G88" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H88" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I88" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J88" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10">
+      <c r="A89" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D89" s="3">
+        <v>45980</v>
+      </c>
+      <c r="E89" s="3">
+        <v>45980</v>
+      </c>
+      <c r="F89" s="2"/>
+      <c r="G89" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H89" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I89" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J89" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10">
+      <c r="A90" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D90" s="3">
+        <v>45980</v>
+      </c>
+      <c r="E90" s="3">
+        <v>45980</v>
+      </c>
+      <c r="F90" s="2"/>
+      <c r="G90" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H90" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I90" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J90" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10">
+      <c r="A91" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D91" s="3">
+        <v>45973</v>
+      </c>
+      <c r="E91" s="3">
+        <v>45973</v>
+      </c>
+      <c r="F91" s="2"/>
+      <c r="G91" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H91" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I91" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10">
+      <c r="A92" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D92" s="3">
+        <v>45973</v>
+      </c>
+      <c r="E92" s="3">
+        <v>45973</v>
+      </c>
+      <c r="F92" s="2"/>
+      <c r="G92" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H92" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I92" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J92" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10">
+      <c r="A93" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D93" s="3">
+        <v>45973</v>
+      </c>
+      <c r="E93" s="3">
+        <v>45973</v>
+      </c>
+      <c r="F93" s="2"/>
+      <c r="G93" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H93" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I93" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J93" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10">
+      <c r="A94" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D94" s="3">
+        <v>45973</v>
+      </c>
+      <c r="E94" s="3">
+        <v>45980</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G94" s="4">
+        <v>-2916</v>
+      </c>
+      <c r="H94" s="4">
+        <v>-612.36</v>
+      </c>
+      <c r="I94" s="4">
+        <v>-3528.36</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10">
+      <c r="A95" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D95" s="3">
+        <v>45973</v>
+      </c>
+      <c r="E95" s="3">
+        <v>45980</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G95" s="4">
+        <v>-3666</v>
+      </c>
+      <c r="H95" s="4">
+        <v>-769.86</v>
+      </c>
+      <c r="I95" s="4">
+        <v>-4435.86</v>
+      </c>
+      <c r="J95" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10">
+      <c r="A96" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D96" s="3">
+        <v>45967</v>
+      </c>
+      <c r="E96" s="3">
+        <v>45974</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G96" s="4">
+        <v>-3467</v>
+      </c>
+      <c r="H96" s="4">
+        <v>-728.0700000000001</v>
+      </c>
+      <c r="I96" s="4">
+        <v>-4195.07</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10">
+      <c r="A97" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D97" s="3">
+        <v>45966</v>
+      </c>
+      <c r="E97" s="3">
+        <v>45973</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="G97" s="4">
+        <v>-2768</v>
+      </c>
+      <c r="H97" s="4">
+        <v>-581.28</v>
+      </c>
+      <c r="I97" s="4">
+        <v>-3349.28</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10">
+      <c r="A98" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D98" s="3">
+        <v>45966</v>
+      </c>
+      <c r="E98" s="3">
+        <v>45966</v>
+      </c>
+      <c r="F98" s="2"/>
+      <c r="G98" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H98" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I98" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10">
+      <c r="A99" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D99" s="3">
+        <v>45966</v>
+      </c>
+      <c r="E99" s="3">
+        <v>45966</v>
+      </c>
+      <c r="F99" s="2"/>
+      <c r="G99" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H99" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I99" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J99" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10">
+      <c r="A100" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D100" s="3">
+        <v>45966</v>
+      </c>
+      <c r="E100" s="3">
+        <v>45966</v>
+      </c>
+      <c r="F100" s="2"/>
+      <c r="G100" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H100" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I100" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10">
+      <c r="A101" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D101" s="3">
+        <v>45965</v>
+      </c>
+      <c r="E101" s="3">
+        <v>45965</v>
+      </c>
+      <c r="F101" s="2"/>
+      <c r="G101" s="4">
+        <v>-200</v>
+      </c>
+      <c r="H101" s="4">
+        <v>-42</v>
+      </c>
+      <c r="I101" s="4">
+        <v>-242</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10">
+      <c r="A102" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D102" s="3">
+        <v>45964</v>
+      </c>
+      <c r="E102" s="3">
+        <v>45964</v>
+      </c>
+      <c r="F102" s="2"/>
+      <c r="G102" s="4">
+        <v>-100</v>
+      </c>
+      <c r="H102" s="4">
+        <v>-21</v>
+      </c>
+      <c r="I102" s="4">
+        <v>-121</v>
+      </c>
+      <c r="J102" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10">
+      <c r="A103" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D103" s="3">
+        <v>45961</v>
+      </c>
+      <c r="E103" s="3">
+        <v>45961</v>
+      </c>
+      <c r="F103" s="2"/>
+      <c r="G103" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H103" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I103" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J103" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10">
+      <c r="A104" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="D104" s="3">
+        <v>45961</v>
+      </c>
+      <c r="E104" s="3">
+        <v>45961</v>
+      </c>
+      <c r="F104" s="2"/>
+      <c r="G104" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H104" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I104" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J104" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10">
+      <c r="A105" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D105" s="3">
+        <v>45961</v>
+      </c>
+      <c r="E105" s="3">
+        <v>45961</v>
+      </c>
+      <c r="F105" s="2"/>
+      <c r="G105" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="H105" s="4">
+        <v>-20</v>
+      </c>
+      <c r="I105" s="4">
+        <v>-1020</v>
+      </c>
+      <c r="J105" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10">
+      <c r="A106" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D106" s="3">
+        <v>45960</v>
+      </c>
+      <c r="E106" s="3">
+        <v>45960</v>
+      </c>
+      <c r="F106" s="2"/>
+      <c r="G106" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H106" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I106" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J106" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10">
+      <c r="A107" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D107" s="3">
+        <v>45959</v>
+      </c>
+      <c r="E107" s="3">
+        <v>45966</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="G107" s="4">
+        <v>-3102</v>
+      </c>
+      <c r="H107" s="4">
+        <v>-651.42</v>
+      </c>
+      <c r="I107" s="4">
+        <v>-3753.42</v>
+      </c>
+      <c r="J107" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10">
+      <c r="A108" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D108" s="3">
+        <v>45959</v>
+      </c>
+      <c r="E108" s="3">
+        <v>45966</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="G108" s="4">
+        <v>-3757</v>
+      </c>
+      <c r="H108" s="4">
+        <v>-788.97</v>
+      </c>
+      <c r="I108" s="4">
+        <v>-4545.97</v>
+      </c>
+      <c r="J108" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10">
+      <c r="A109" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D109" s="3">
+        <v>45954</v>
+      </c>
+      <c r="E109" s="3">
+        <v>45954</v>
+      </c>
+      <c r="F109" s="2"/>
+      <c r="G109" s="4">
+        <v>-1</v>
+      </c>
+      <c r="H109" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="I109" s="4">
+        <v>-1.21</v>
+      </c>
+      <c r="J109" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10">
+      <c r="A110" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D110" s="3">
+        <v>45953</v>
+      </c>
+      <c r="E110" s="3">
+        <v>45960</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="G110" s="4">
+        <v>-3461</v>
+      </c>
+      <c r="H110" s="4">
+        <v>-726.8099999999999</v>
+      </c>
+      <c r="I110" s="4">
+        <v>-4187.81</v>
+      </c>
+      <c r="J110" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10">
+      <c r="A111" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D111" s="3">
+        <v>45953</v>
+      </c>
+      <c r="E111" s="3">
+        <v>45960</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="G111" s="4">
+        <v>-2936</v>
+      </c>
+      <c r="H111" s="4">
+        <v>-616.5599999999999</v>
+      </c>
+      <c r="I111" s="4">
+        <v>-3552.56</v>
+      </c>
+      <c r="J111" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10">
+      <c r="A112" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D112" s="3">
+        <v>45947</v>
+      </c>
+      <c r="E112" s="3">
+        <v>45954</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="G112" s="4">
+        <v>-874</v>
+      </c>
+      <c r="H112" s="4">
+        <v>-183.54</v>
+      </c>
+      <c r="I112" s="4">
+        <v>-1057.54</v>
+      </c>
+      <c r="J112" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10">
+      <c r="A113" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D113" s="3">
+        <v>45947</v>
+      </c>
+      <c r="E113" s="3">
+        <v>45954</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G113" s="4">
+        <v>-1007</v>
+      </c>
+      <c r="H113" s="4">
+        <v>-211.47</v>
+      </c>
+      <c r="I113" s="4">
+        <v>-1218.47</v>
+      </c>
+      <c r="J113" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10">
+      <c r="A114" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D114" s="3">
+        <v>45935</v>
+      </c>
+      <c r="E114" s="3">
+        <v>45935</v>
+      </c>
+      <c r="F114" s="2"/>
+      <c r="G114" s="4">
+        <v>-46.67</v>
+      </c>
+      <c r="H114" s="4">
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="I114" s="4">
+        <v>-56.47</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10">
+      <c r="A115" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D115" s="3">
+        <v>45934</v>
+      </c>
+      <c r="E115" s="3">
+        <v>45934</v>
+      </c>
+      <c r="F115" s="2"/>
+      <c r="G115" s="4">
+        <v>-20</v>
+      </c>
+      <c r="H115" s="4">
+        <v>-4.2</v>
+      </c>
+      <c r="I115" s="4">
+        <v>-24.2</v>
+      </c>
+      <c r="J115" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10">
+      <c r="A116" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D116" s="3">
+        <v>45931</v>
+      </c>
+      <c r="E116" s="3">
+        <v>45931</v>
+      </c>
+      <c r="F116" s="2"/>
+      <c r="G116" s="4">
+        <v>-100</v>
+      </c>
+      <c r="H116" s="4">
+        <v>-2</v>
+      </c>
+      <c r="I116" s="4">
+        <v>-102</v>
+      </c>
+      <c r="J116" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>